<commit_message>
Add brands/footer to store onboarding system
- Add Brands tab to spreadsheet template (brand name + logo file)
- Add Footer Text field to Store Info tab
- Conversion script now generates footer HTML with brand logos
- --output-html mode replaces the footer in generated index.html
- Updated Drive folder README to include brand logo uploads

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/onboarding/DreamFinder_Onboarding_Template.xlsx
+++ b/onboarding/DreamFinder_Onboarding_Template.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Store Info" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Mattresses" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Accessories" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Feature Keywords" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Instructions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Brands" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Feature Keywords" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Instructions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -505,6 +506,7 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,6 +565,11 @@
           <t>Contact Email</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Footer Text</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -616,6 +623,11 @@
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>sleep@belfurniture.com</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Powered by DreamFinder · (c) 2026 Bel Furniture</t>
         </is>
       </c>
     </row>
@@ -631,6 +643,7 @@
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1278,470 +1291,59 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Feature Keyword</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>What It Means / When to Use</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Quiz Connection</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Brand Name *</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Logo File Name *
+(e.g. restonic-logo.png)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>plush</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>Very soft feel (firmness 1-3)</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Matches side sleepers, lighter body types</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Restonic</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>restonic-logo.png</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Moderate feel (firmness 4-6)</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Most versatile — matches combo sleepers, average body types</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Spring Air</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>springair-logo.png</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>firm</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Hard feel (firmness 7-10)</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Matches back/stomach sleepers, heavier body types</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>cooling</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Has cooling technology (gel, phase-change, copper)</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Matches hot sleepers, temperature complaints</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>support</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Strong core support system</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Matches back pain, heavier body types</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>hybrid</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Coils + foam construction</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>General positive scoring — most versatile type</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>innerspring</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Traditional coil construction</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Budget-friendly, good support</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>latex</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Contains latex foam layers</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Natural feel, responsive, hypoallergenic</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>responsive</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Quick response to movement (not slow-sinking)</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Combo sleepers, people who move a lot</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>pressure-relief</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Relieves pressure points (hips, shoulders)</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Side sleepers, joint pain, shoulder issues</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>motion-isolation</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Minimizes partner movement transfer</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Couples, light sleepers with partners</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>hand-tufting</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Hand-tufted construction (premium)</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Premium/durability seekers</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>copper</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Copper-infused materials</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Antimicrobial, cooling, wellness-focused</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>gel-memory-foam</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Gel-infused memory foam</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Cooling + pressure relief</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>gel-infused-foam</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Gel-infused foam (non-memory)</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Cooling + comfort</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>serene-foam</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Serene foam comfort layer</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Comfort + cooling</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>foam-encasement</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Foam-encased edge support</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Edge support, full sleep surface</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>back-supporter-technology</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Back Supporter certified</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Back pain sufferers</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>quality</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>High-quality materials/construction</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Durability seekers</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>comfort</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>General comfort emphasis</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Broad appeal</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>lifetime-warranty</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Comes with lifetime warranty</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Durability/value seekers</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>anti-viral</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Antiviral material properties</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Health-conscious sleepers</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>anti-bacterial</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Antibacterial material properties</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Health-conscious sleepers</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>anti-microbial</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Antimicrobial material properties</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Health-conscious sleepers</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>anti-inflammatory</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>Anti-inflammatory material properties</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Health-conscious sleepers</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>durability</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Built to last / premium construction</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Long-term investment seekers</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Bel-O-Pedic</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>belopedic-logo.png</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1358,485 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Feature Keyword</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>What It Means / When to Use</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Quiz Connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>plush</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Very soft feel (firmness 1-3)</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Matches side sleepers, lighter body types</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Moderate feel (firmness 4-6)</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Most versatile — matches combo sleepers, average body types</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Hard feel (firmness 7-10)</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Matches back/stomach sleepers, heavier body types</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>cooling</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Has cooling technology (gel, phase-change, copper)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Matches hot sleepers, temperature complaints</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>support</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Strong core support system</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Matches back pain, heavier body types</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Coils + foam construction</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>General positive scoring — most versatile type</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>innerspring</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Traditional coil construction</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Budget-friendly, good support</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>latex</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Contains latex foam layers</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Natural feel, responsive, hypoallergenic</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>responsive</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Quick response to movement (not slow-sinking)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Combo sleepers, people who move a lot</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>pressure-relief</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Relieves pressure points (hips, shoulders)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Side sleepers, joint pain, shoulder issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>motion-isolation</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Minimizes partner movement transfer</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Couples, light sleepers with partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>hand-tufting</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Hand-tufted construction (premium)</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Premium/durability seekers</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Copper-infused materials</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Antimicrobial, cooling, wellness-focused</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>gel-memory-foam</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Gel-infused memory foam</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Cooling + pressure relief</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>gel-infused-foam</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Gel-infused foam (non-memory)</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Cooling + comfort</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>serene-foam</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Serene foam comfort layer</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Comfort + cooling</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>foam-encasement</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Foam-encased edge support</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Edge support, full sleep surface</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>back-supporter-technology</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Back Supporter certified</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Back pain sufferers</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>quality</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>High-quality materials/construction</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Durability seekers</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>comfort</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>General comfort emphasis</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Broad appeal</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>lifetime-warranty</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Comes with lifetime warranty</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Durability/value seekers</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>anti-viral</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Antiviral material properties</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Health-conscious sleepers</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>anti-bacterial</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Antibacterial material properties</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Health-conscious sleepers</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>anti-microbial</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Antimicrobial material properties</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Health-conscious sleepers</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>anti-inflammatory</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Anti-inflammatory material properties</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Health-conscious sleepers</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>durability</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Built to last / premium construction</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Long-term investment seekers</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1994,109 +2074,140 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>STEP 4: UPLOAD IMAGES TO THE SHARED DRIVE FOLDER</t>
+          <t>STEP 4: BRANDS TAB</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Place your files in the shared Google Drive folder:</t>
+          <t>Add one row per mattress brand you carry. These appear in the app footer.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  logos/        — Your store logo + square PWA icons (192x192 and 512x512)</t>
+          <t>• Brand Name — The display name (e.g., 'Serta', 'Sealy').</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  mattresses/   — One image per mattress, named to match the ID column (e.g., athena.png)</t>
+          <t>• Logo File Name — Must match a file in the logos/ folder (e.g., serta-logo.png).</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  accessories/  — One image per accessory, named to match the ID column (e.g., base-bt3000.jpg)</t>
-        </is>
-      </c>
+      <c r="A40" s="10" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr"/>
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>STEP 5: UPLOAD IMAGES TO THE SHARED DRIVE FOLDER</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr">
-        <is>
-          <t>IMAGE REQUIREMENTS:</t>
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Place your files in the shared Google Drive folder:</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Mattresses:  600×400px recommended, PNG or JPG, transparent background preferred</t>
+          <t xml:space="preserve">  logos/        — Your store logo, PWA icons (192x192 and 512x512), and brand logos</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accessories: 400×300px recommended, PNG, JPG, or WebP</t>
+          <t xml:space="preserve">  mattresses/   — One image per mattress, named to match the ID column (e.g., athena.png)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Logo:        Min 400px wide, transparent background (PNG)</t>
+          <t xml:space="preserve">  accessories/  — One image per accessory, named to match the ID column (e.g., base-bt3000.jpg)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PWA Icons:   Exactly 192×192 and 512×512 pixels, square, PNG</t>
-        </is>
-      </c>
+      <c r="A46" s="10" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="inlineStr"/>
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>IMAGE REQUIREMENTS:</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="inlineStr">
-        <is>
-          <t>TIPS:</t>
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Mattresses:  600×400px recommended, PNG or JPG, transparent background preferred</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>• The YELLOW example rows show Bel Furniture's data — delete them before submitting.</t>
+          <t xml:space="preserve">  Accessories: 400×300px recommended, PNG, JPG, or WebP</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>• Use the Feature Keywords tab as a reference when filling in feature keywords.</t>
+          <t xml:space="preserve">  Logo:        Min 400px wide, transparent background (PNG)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">  PWA Icons:   Exactly 192×192 and 512×512 pixels, square, PNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>TIPS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>• The YELLOW example rows show Bel Furniture's data — delete them before submitting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>• Use the Feature Keywords tab as a reference when filling in feature keywords.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
           <t>• You can add your OWN feature keywords if needed — just be consistent.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>• If you're unsure about match scores for accessories, leave them blank and we'll help.</t>
         </is>

</xml_diff>

<commit_message>
Add optional PWA icon generation pipeline
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/onboarding/DreamFinder_Onboarding_Template.xlsx
+++ b/onboarding/DreamFinder_Onboarding_Template.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF1"/>
+  <dimension ref="A1:BG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -526,6 +526,7 @@
     <col width="20" customWidth="1" min="56" max="56"/>
     <col width="22" customWidth="1" min="57" max="57"/>
     <col width="27" customWidth="1" min="58" max="58"/>
+    <col width="15" customWidth="1" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -817,6 +818,11 @@
       <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Manifest Background Color</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>App Icon File</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A48"/>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1707,24 +1713,45 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr"/>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  App Icon File (Store Info, optional): a single square PNG (&gt;=512px) in the</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>NEED A FILLED EXAMPLE?</t>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  logos/ image folder. When set, the pipeline generates the installable-app</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">  (PWA) icons. Leave blank to skip - the app still works without it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>NEED A FILLED EXAMPLE?</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  The Bel Furniture fixture is the worked, fully-filled example. This template</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  is intentionally blank.</t>
         </is>

</xml_diff>